<commit_message>
Refactor NAMESPACE and R scripts for improved function exports and documentation; add new function to import OFX data; update r_inad function for better data handling; create new Excel files for data processing.
</commit_message>
<xml_diff>
--- a/dados/Estação - status 2025_05_30.xlsx
+++ b/dados/Estação - status 2025_05_30.xlsx
@@ -1164,4 +1164,231 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006C56FB2846673243A9735D5EC6051572" ma:contentTypeVersion="11" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="36569ac63cfce8ff0f8884bc80e67f1c">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5a5f483f-f768-438e-b4ef-63f46a7558dd" xmlns:ns3="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2040da04b75a9ea4fe796fa8180f8ca6" ns2:_="" ns3:_="">
+    <xsd:import namespace="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
+    <xsd:import namespace="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="5a5f483f-f768-438e-b4ef-63f46a7558dd" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Marcações de imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="d52aaf24-8448-430e-97e8-d28c57d898a4" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{6bacedc3-d3dc-49dd-a723-47ba9b97a11c}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="dd8c73df-45bd-468c-aae5-f3faedcbd5e2">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de Conteúdo"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a5f483f-f768-438e-b4ef-63f46a7558dd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20178032-B2A6-4FCC-91F0-8DF750D636F9}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE9ACA24-D917-479C-A1E1-7B2CA9564B5D}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D40DE643-D85C-4163-8142-2F4E4A8CDD77}"/>
 </file>
</xml_diff>

<commit_message>
Add new Excel files for various car data spanning from 2025 to 2099
- Added car_AMP-20250901_20991231.xlsx
- Added car_AVS-20250901_20991231.xlsx
- Added car_GRA-20250901_20991231.xlsx
- Added car_LUC-20250901_20991231.xlsx
- Added car_POM-20250901_20991231.xlsx
- Added car_SN2-20250901_20991231.xlsx
- Added car_SN4-20250901_20991231.xlsx
</commit_message>
<xml_diff>
--- a/dados/Estação - status 2025_05_30.xlsx
+++ b/dados/Estação - status 2025_05_30.xlsx
@@ -1,25 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://incorporadoraampla-my.sharepoint.com/personal/vitor_amplaincorporadora_com_br/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://incorporadoraampla.sharepoint.com/sites/Controladoria/Documentos Compartilhados/amplaGitHub/dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="255" documentId="8_{C0F877D4-A7C2-4284-928E-04C8FFFB6007}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E581BFD-7B85-43A0-A6D4-40094D200B3C}"/>
+  <xr:revisionPtr revIDLastSave="257" documentId="8_{C0F877D4-A7C2-4284-928E-04C8FFFB6007}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC741642-C409-4056-849A-A0B48DF6F2E6}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{240890F9-D451-4B7D-B96D-9A56BDF9E0C9}"/>
+    <workbookView xWindow="20370" yWindow="-8025" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{240890F9-D451-4B7D-B96D-9A56BDF9E0C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Estação" sheetId="1" r:id="rId1"/>
     <sheet name="Planilha4" sheetId="4" r:id="rId2"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId3"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -238,14 +236,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -283,50 +280,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="DRE Finc"/>
-      <sheetName val="Demonstrativo Eco-Finc"/>
-      <sheetName val="Fluxo"/>
-      <sheetName val="Matriz MCMV"/>
-      <sheetName val="Matriz"/>
-      <sheetName val="CurvaObra"/>
-      <sheetName val="CurvaVenda"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="34">
-          <cell r="E34">
-            <v>58847199.720000006</v>
-          </cell>
-        </row>
-        <row r="76">
-          <cell r="E76">
-            <v>56633497.8864685</v>
-          </cell>
-        </row>
-        <row r="79">
-          <cell r="E79">
-            <v>34309815.140000001</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -660,7 +613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A38821AB-3D55-4EC7-97EA-6560C36FE8E7}">
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
@@ -670,7 +623,7 @@
     <col min="7" max="7" width="16.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>23</v>
       </c>
@@ -681,14 +634,8 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
@@ -699,14 +646,8 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>11</v>
       </c>
@@ -719,41 +660,41 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
       <c r="B4" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="6">
         <v>40458120</v>
       </c>
       <c r="G4" s="1"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
       <c r="B5" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="6">
         <v>37884983.57</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
       <c r="B6" t="s">
         <v>0</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="9">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -764,7 +705,7 @@
         <v>29209178.98</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -775,7 +716,7 @@
         <v>2045373.9</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -786,7 +727,7 @@
         <v>15862</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -797,7 +738,7 @@
         <v>5388898.2599999998</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -808,17 +749,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="2"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="8">
         <f>SUM(C19:C20)</f>
         <v>71596281.780000001</v>
       </c>
@@ -839,7 +780,7 @@
       <c r="F18" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G18" s="7">
+      <c r="G18" s="6">
         <v>13649530.609999999</v>
       </c>
     </row>
@@ -866,10 +807,10 @@
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="8" t="s">
+      <c r="A23" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="9">
+      <c r="B23" s="8">
         <f>SUM(C25:C28)</f>
         <v>18489153.759999998</v>
       </c>
@@ -884,10 +825,9 @@
       <c r="C24" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D24" s="6"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
+      <c r="A25" t="s">
         <v>15</v>
       </c>
       <c r="B25" t="s">
@@ -896,8 +836,6 @@
       <c r="C25" s="1">
         <v>5388898.2599999998</v>
       </c>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
@@ -950,19 +888,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="11" t="s">
         <v>11</v>
       </c>
     </row>
@@ -970,8 +908,7 @@
       <c r="A2" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="11">
-        <f>'[1]Demonstrativo Eco-Finc'!$E$34</f>
+      <c r="B2" s="10">
         <v>58847199.720000006</v>
       </c>
       <c r="C2" t="s">
@@ -1005,7 +942,7 @@
       <c r="A4" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="10">
         <v>7034961.9199999999</v>
       </c>
       <c r="C4" t="s">
@@ -1056,7 +993,7 @@
       <c r="A7" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="10">
         <v>24235452.960000001</v>
       </c>
       <c r="C7" t="s">
@@ -1073,7 +1010,7 @@
       <c r="A8" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="10">
         <v>3834818</v>
       </c>
       <c r="C8" t="s">
@@ -1090,7 +1027,7 @@
       <c r="A9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="10">
         <f>13794448.52-B8</f>
         <v>9959630.5199999996</v>
       </c>
@@ -1108,8 +1045,7 @@
       <c r="A10" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="11">
-        <f>'[1]Demonstrativo Eco-Finc'!$E$79-B8</f>
+      <c r="B10" s="10">
         <v>30474997.140000001</v>
       </c>
       <c r="C10" t="s">
@@ -1126,8 +1062,7 @@
       <c r="A11" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B11" s="11">
-        <f>'[1]Demonstrativo Eco-Finc'!$E$76-'[1]Demonstrativo Eco-Finc'!$E$79-B9</f>
+      <c r="B11" s="10">
         <v>12364052.2264685</v>
       </c>
       <c r="C11" t="s">
@@ -1144,7 +1079,7 @@
       <c r="A12" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="10">
         <f>SUM(B3:B7)-SUM(B8:B11)</f>
         <v>33451937.653531492</v>
       </c>
@@ -1362,15 +1297,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a5f483f-f768-438e-b4ef-63f46a7558dd">
@@ -1381,14 +1307,49 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20178032-B2A6-4FCC-91F0-8DF750D636F9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20178032-B2A6-4FCC-91F0-8DF750D636F9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
+    <ds:schemaRef ds:uri="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE9ACA24-D917-479C-A1E1-7B2CA9564B5D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D40DE643-D85C-4163-8142-2F4E4A8CDD77}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
+    <ds:schemaRef ds:uri="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D40DE643-D85C-4163-8142-2F4E4A8CDD77}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE9ACA24-D917-479C-A1E1-7B2CA9564B5D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>